<commit_message>
Datei auf Sektion Trier angepasst
</commit_message>
<xml_diff>
--- a/Keys.xlsx
+++ b/Keys.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Berenike\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DA9DE4A-9E69-43C2-A11C-02AEDB90E01B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9038FD3A-40B7-4EC7-A950-822AD82E6884}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Kategorie" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="70">
   <si>
     <t>ID</t>
   </si>
@@ -43,132 +43,39 @@
     <t>ShortCode</t>
   </si>
   <si>
-    <t>Bergwanderung/Bergtour</t>
-  </si>
-  <si>
     <t>BW</t>
   </si>
   <si>
-    <t>Hochtour</t>
-  </si>
-  <si>
     <t>HT</t>
   </si>
   <si>
     <t>Bouldern</t>
   </si>
   <si>
-    <t>BO</t>
-  </si>
-  <si>
-    <t>Sportklettern</t>
-  </si>
-  <si>
-    <t>KL</t>
-  </si>
-  <si>
-    <t>Klettersteigtour</t>
-  </si>
-  <si>
     <t>KS</t>
   </si>
   <si>
-    <t>Mountainbiketour</t>
-  </si>
-  <si>
     <t>MTB</t>
   </si>
   <si>
-    <t>Schneeschuhtour</t>
-  </si>
-  <si>
     <t>SSG</t>
   </si>
   <si>
-    <t>Freeride</t>
-  </si>
-  <si>
-    <t>FR</t>
-  </si>
-  <si>
     <t>Skilanglauf</t>
   </si>
   <si>
-    <t>SL</t>
-  </si>
-  <si>
     <t>Skitour</t>
   </si>
   <si>
     <t>ST</t>
   </si>
   <si>
-    <t>Trailrunning/Berglauf</t>
-  </si>
-  <si>
-    <t>TR</t>
-  </si>
-  <si>
-    <t>Snowboard</t>
-  </si>
-  <si>
-    <t>SN</t>
-  </si>
-  <si>
-    <t>Skigymnastik</t>
-  </si>
-  <si>
-    <t>SG</t>
-  </si>
-  <si>
-    <t>Skifahren</t>
-  </si>
-  <si>
     <t>SKI</t>
   </si>
   <si>
     <t>Wandern</t>
   </si>
   <si>
-    <t>WA</t>
-  </si>
-  <si>
-    <t>Kinder</t>
-  </si>
-  <si>
-    <t>KI</t>
-  </si>
-  <si>
-    <t>Yoga</t>
-  </si>
-  <si>
-    <t>YO</t>
-  </si>
-  <si>
-    <t>Familien</t>
-  </si>
-  <si>
-    <t>FA</t>
-  </si>
-  <si>
-    <t>Natur</t>
-  </si>
-  <si>
-    <t>NAT</t>
-  </si>
-  <si>
-    <t>Alpinklettern</t>
-  </si>
-  <si>
-    <t>AK</t>
-  </si>
-  <si>
-    <t>Senior*innen</t>
-  </si>
-  <si>
-    <t>SEN</t>
-  </si>
-  <si>
     <t>Skihochtour</t>
   </si>
   <si>
@@ -178,21 +85,6 @@
     <t>Radtour</t>
   </si>
   <si>
-    <t>RAD</t>
-  </si>
-  <si>
-    <t>Eisklettern</t>
-  </si>
-  <si>
-    <t>EKL</t>
-  </si>
-  <si>
-    <t>Nordic Walking</t>
-  </si>
-  <si>
-    <t>NW</t>
-  </si>
-  <si>
     <t>leicht</t>
   </si>
   <si>
@@ -271,9 +163,6 @@
     <t>lastName</t>
   </si>
   <si>
-    <t>/267 - Sektion Turner-Alpenkränzchen/Personen/Personen/Max Mustermann</t>
-  </si>
-  <si>
     <t>Max</t>
   </si>
   <si>
@@ -283,63 +172,9 @@
     <t>Gruppe</t>
   </si>
   <si>
-    <t>Allgemein</t>
-  </si>
-  <si>
-    <t>/267 - Sektion Turner-Alpenkränzchen/Gruppen/Allgemein</t>
-  </si>
-  <si>
-    <t>TAK</t>
-  </si>
-  <si>
     <t>Mountainbike</t>
   </si>
   <si>
-    <t>/267 - Sektion Turner-Alpenkränzchen/Gruppen/Mountainbike</t>
-  </si>
-  <si>
-    <t>Mankeis</t>
-  </si>
-  <si>
-    <t>/267 - Sektion Turner-Alpenkränzchen/Gruppen/Kinder- Jugend- und Familiengruppen/Mankeis</t>
-  </si>
-  <si>
-    <t>MANK</t>
-  </si>
-  <si>
-    <t>Jugendklettergruppe</t>
-  </si>
-  <si>
-    <t>/267 - Sektion Turner-Alpenkränzchen/Gruppen/Kinder- Jugend- und Familiengruppen/Jugendklettergruppe</t>
-  </si>
-  <si>
-    <t>JUK</t>
-  </si>
-  <si>
-    <t>Familiengruppe</t>
-  </si>
-  <si>
-    <t>/267 - Sektion Turner-Alpenkränzchen/Gruppen/Kinder- Jugend- und Familiengruppen/Familiengruppe</t>
-  </si>
-  <si>
-    <t>FAM</t>
-  </si>
-  <si>
-    <t>Klettertreff</t>
-  </si>
-  <si>
-    <t>/267 - Sektion Turner-Alpenkränzchen/Gruppen/Klettertreff</t>
-  </si>
-  <si>
-    <t>KLT</t>
-  </si>
-  <si>
-    <t>Seniorengruppe</t>
-  </si>
-  <si>
-    <t>/267 - Sektion Turner-Alpenkränzchen/Gruppen/Seniorengruppe</t>
-  </si>
-  <si>
     <t>Bergsteigen</t>
   </si>
   <si>
@@ -364,14 +199,56 @@
     <t>Wettkampf</t>
   </si>
   <si>
-    <t>HAT</t>
+    <t>WAN</t>
+  </si>
+  <si>
+    <t>RT</t>
+  </si>
+  <si>
+    <t>SLL</t>
+  </si>
+  <si>
+    <t>WK</t>
+  </si>
+  <si>
+    <t>BS</t>
+  </si>
+  <si>
+    <t>BOU</t>
+  </si>
+  <si>
+    <t>KLE</t>
+  </si>
+  <si>
+    <t>/264 - Sektion Trier/Personen/Personen/Max Mustermann</t>
+  </si>
+  <si>
+    <t>Sonntagswanderung</t>
+  </si>
+  <si>
+    <t>U12-Wanderung</t>
+  </si>
+  <si>
+    <t>Familienwanderung</t>
+  </si>
+  <si>
+    <t>/267 - Sektion Trier/Gruppen/Wandergruppe</t>
+  </si>
+  <si>
+    <t>/267 - Sektion Trier/Gruppen/Mountainbiken</t>
+  </si>
+  <si>
+    <t>WAG</t>
+  </si>
+  <si>
+    <t>MTG</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -398,12 +275,6 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -425,7 +296,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -451,9 +322,6 @@
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -720,7 +588,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F1048576"/>
+  <dimension ref="A1:C1048576"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.44140625" style="3"/>
@@ -729,7 +597,7 @@
     <col min="4" max="4" width="16.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -740,378 +608,212 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A2" s="3">
-        <v>68695</v>
-      </c>
-      <c r="B2" s="6" t="s">
+    <row r="2" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>417</v>
+      </c>
+      <c r="B2" t="s">
+        <v>47</v>
+      </c>
+      <c r="C2" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>418</v>
+      </c>
+      <c r="B3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C3" t="s">
         <v>3</v>
       </c>
-      <c r="C2" t="s">
+    </row>
+    <row r="4" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>419</v>
+      </c>
+      <c r="B4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>420</v>
+      </c>
+      <c r="B5" t="s">
+        <v>49</v>
+      </c>
+      <c r="C5" t="s">
         <v>4</v>
       </c>
-      <c r="D2" t="s">
-        <v>102</v>
-      </c>
-      <c r="E2">
-        <v>417</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A3" s="3">
-        <v>20976</v>
-      </c>
-      <c r="B3" s="6" t="s">
-        <v>5</v>
-      </c>
-      <c r="C3" t="s">
+    </row>
+    <row r="6" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>421</v>
+      </c>
+      <c r="B6" t="s">
+        <v>50</v>
+      </c>
+      <c r="C6" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>422</v>
+      </c>
+      <c r="B7" t="s">
+        <v>51</v>
+      </c>
+      <c r="C7" t="s">
         <v>6</v>
       </c>
-      <c r="D3" t="s">
-        <v>103</v>
-      </c>
-      <c r="E3">
-        <v>418</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A4" s="3">
-        <v>20978</v>
-      </c>
-      <c r="B4" s="6" t="s">
+    </row>
+    <row r="8" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>423</v>
+      </c>
+      <c r="B8" t="s">
+        <v>46</v>
+      </c>
+      <c r="C8" t="s">
         <v>7</v>
       </c>
-      <c r="C4" t="s">
+    </row>
+    <row r="9" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>35246</v>
+      </c>
+      <c r="B9" t="s">
+        <v>16</v>
+      </c>
+      <c r="C9" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>424</v>
+      </c>
+      <c r="B10" t="s">
+        <v>52</v>
+      </c>
+      <c r="C10" t="s">
         <v>8</v>
       </c>
-      <c r="D4" t="s">
-        <v>7</v>
-      </c>
-      <c r="E4">
-        <v>419</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A5" s="3">
-        <v>20979</v>
-      </c>
-      <c r="B5" s="6" t="s">
+    </row>
+    <row r="11" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>871</v>
+      </c>
+      <c r="B11" t="s">
+        <v>53</v>
+      </c>
+      <c r="C11" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>22965</v>
+      </c>
+      <c r="B12" t="s">
+        <v>14</v>
+      </c>
+      <c r="C12" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>425</v>
+      </c>
+      <c r="B13" t="s">
         <v>9</v>
       </c>
-      <c r="C5" t="s">
+      <c r="C13" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>426</v>
+      </c>
+      <c r="B14" t="s">
         <v>10</v>
       </c>
-      <c r="D5" t="s">
-        <v>104</v>
-      </c>
-      <c r="E5">
-        <v>420</v>
-      </c>
-      <c r="F5" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A6" s="3">
-        <v>20980</v>
-      </c>
-      <c r="B6" s="6" t="s">
+      <c r="C14" t="s">
         <v>11</v>
       </c>
-      <c r="C6" t="s">
-        <v>12</v>
-      </c>
-      <c r="D6" t="s">
-        <v>105</v>
-      </c>
-      <c r="E6">
-        <v>421</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A7" s="3">
-        <v>20981</v>
-      </c>
-      <c r="B7" s="6" t="s">
+    </row>
+    <row r="15" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>2284</v>
+      </c>
+      <c r="B15" t="s">
         <v>13</v>
       </c>
-      <c r="C7" t="s">
-        <v>14</v>
-      </c>
-      <c r="D7" t="s">
-        <v>106</v>
-      </c>
-      <c r="E7">
-        <v>422</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A8" s="3">
-        <v>20982</v>
-      </c>
-      <c r="B8" s="6" t="s">
-        <v>15</v>
-      </c>
-      <c r="C8" t="s">
-        <v>16</v>
-      </c>
-      <c r="D8" t="s">
-        <v>86</v>
-      </c>
-      <c r="E8">
-        <v>423</v>
-      </c>
-      <c r="F8" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A9" s="3">
-        <v>20983</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="C9" t="s">
-        <v>18</v>
-      </c>
-      <c r="D9" t="s">
-        <v>47</v>
-      </c>
-      <c r="E9">
-        <v>35246</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A10" s="3">
-        <v>20984</v>
-      </c>
-      <c r="B10" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="C10" t="s">
-        <v>20</v>
-      </c>
-      <c r="D10" t="s">
-        <v>107</v>
-      </c>
-      <c r="E10">
-        <v>424</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A11" s="3">
-        <v>426</v>
-      </c>
-      <c r="B11" s="6" t="s">
-        <v>21</v>
-      </c>
-      <c r="C11" t="s">
-        <v>22</v>
-      </c>
-      <c r="D11" t="s">
-        <v>108</v>
-      </c>
-      <c r="E11">
-        <v>871</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A12" s="3">
-        <v>20986</v>
-      </c>
-      <c r="B12" s="6" t="s">
-        <v>23</v>
-      </c>
-      <c r="C12" t="s">
-        <v>24</v>
-      </c>
-      <c r="D12" t="s">
-        <v>45</v>
-      </c>
-      <c r="E12">
-        <v>22965</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A13" s="3">
-        <v>31791</v>
-      </c>
-      <c r="B13" s="6" t="s">
-        <v>25</v>
-      </c>
-      <c r="C13" t="s">
-        <v>26</v>
-      </c>
-      <c r="D13" t="s">
-        <v>19</v>
-      </c>
-      <c r="E13">
-        <v>425</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A14" s="3">
-        <v>31792</v>
-      </c>
-      <c r="B14" s="6" t="s">
-        <v>27</v>
-      </c>
-      <c r="C14" t="s">
-        <v>28</v>
-      </c>
-      <c r="D14" t="s">
-        <v>21</v>
-      </c>
-      <c r="E14">
-        <v>426</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A15" s="3">
-        <v>32221</v>
-      </c>
-      <c r="B15" s="6" t="s">
-        <v>29</v>
-      </c>
       <c r="C15" t="s">
-        <v>30</v>
-      </c>
-      <c r="D15" t="s">
-        <v>31</v>
-      </c>
-      <c r="E15">
-        <v>2284</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A16" s="3">
-        <v>32222</v>
-      </c>
-      <c r="B16" s="12" t="s">
-        <v>31</v>
+        <v>55</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>39348</v>
+      </c>
+      <c r="B16" t="s">
+        <v>54</v>
       </c>
       <c r="C16" t="s">
-        <v>32</v>
-      </c>
-      <c r="D16" t="s">
-        <v>109</v>
-      </c>
-      <c r="E16">
-        <v>39348</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A17" s="3">
-        <v>32223</v>
-      </c>
-      <c r="B17" s="6" t="s">
-        <v>33</v>
-      </c>
-      <c r="C17" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A18" s="3">
-        <v>32247</v>
-      </c>
-      <c r="B18" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="C18" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A19" s="3">
-        <v>32277</v>
-      </c>
-      <c r="B19" s="6" t="s">
-        <v>37</v>
-      </c>
-      <c r="C19" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A20" s="3">
-        <v>45911</v>
-      </c>
-      <c r="B20" s="6" t="s">
-        <v>39</v>
-      </c>
-      <c r="C20" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A21" s="3">
-        <v>47973</v>
-      </c>
-      <c r="B21" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="C21" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A22" s="3">
-        <v>48021</v>
-      </c>
-      <c r="B22" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="C22" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A23" s="3">
-        <v>51837</v>
-      </c>
-      <c r="B23" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="C23" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A24" s="3">
-        <v>71574</v>
-      </c>
-      <c r="B24" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="C24" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A25" s="3">
-        <v>76043</v>
-      </c>
-      <c r="B25" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="C25" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A26" s="3">
-        <v>76045</v>
-      </c>
-      <c r="B26" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="C26" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A17"/>
+      <c r="B17"/>
+    </row>
+    <row r="18" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A18"/>
+      <c r="B18"/>
+    </row>
+    <row r="19" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A19"/>
+      <c r="B19"/>
+    </row>
+    <row r="20" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A20"/>
+      <c r="B20"/>
+    </row>
+    <row r="21" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A21"/>
+      <c r="B21"/>
+    </row>
+    <row r="22" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A22"/>
+      <c r="B22"/>
+    </row>
+    <row r="23" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A23"/>
+      <c r="B23"/>
+    </row>
+    <row r="24" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A24"/>
+      <c r="B24"/>
+    </row>
+    <row r="25" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A25"/>
+      <c r="B25"/>
+    </row>
+    <row r="26" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A26"/>
+      <c r="B26"/>
+    </row>
+    <row r="27" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B27"/>
     </row>
     <row r="1048574" ht="14.4" x14ac:dyDescent="0.3"/>
@@ -1149,7 +851,7 @@
         <v>413</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>53</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1157,7 +859,7 @@
         <v>414</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>54</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1165,7 +867,7 @@
         <v>415</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>55</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1173,7 +875,7 @@
         <v>416</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>56</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -1208,7 +910,7 @@
         <v>409</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>57</v>
+        <v>21</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1216,7 +918,7 @@
         <v>410</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>54</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1224,7 +926,7 @@
         <v>411</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>58</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1232,7 +934,7 @@
         <v>412</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>59</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -1267,7 +969,7 @@
         <v>405</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>60</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1275,7 +977,7 @@
         <v>406</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>61</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1283,7 +985,7 @@
         <v>407</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>62</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1291,7 +993,7 @@
         <v>408</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>63</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>
@@ -1325,17 +1027,17 @@
       <c r="A2" s="3">
         <v>392</v>
       </c>
-      <c r="B2" s="13" t="s">
-        <v>64</v>
-      </c>
-      <c r="C2" s="13"/>
+      <c r="B2" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" s="12"/>
     </row>
     <row r="3" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A3" s="3">
         <v>393</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>65</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
@@ -1343,7 +1045,7 @@
         <v>394</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>66</v>
+        <v>30</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
@@ -1351,7 +1053,7 @@
         <v>395</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>67</v>
+        <v>31</v>
       </c>
     </row>
     <row r="6" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
@@ -1359,7 +1061,7 @@
         <v>396</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>68</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
@@ -1367,7 +1069,7 @@
         <v>48744</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>69</v>
+        <v>33</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
@@ -1375,7 +1077,7 @@
         <v>48745</v>
       </c>
       <c r="B8" t="s">
-        <v>70</v>
+        <v>34</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
@@ -1383,7 +1085,7 @@
         <v>48746</v>
       </c>
       <c r="B9" t="s">
-        <v>71</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -1421,7 +1123,7 @@
         <v>397</v>
       </c>
       <c r="B2" t="s">
-        <v>72</v>
+        <v>36</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1429,7 +1131,7 @@
         <v>398</v>
       </c>
       <c r="B3" t="s">
-        <v>73</v>
+        <v>37</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1437,7 +1139,7 @@
         <v>39481</v>
       </c>
       <c r="B4" t="s">
-        <v>74</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -1462,16 +1164,16 @@
   <sheetData>
     <row r="1" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
-        <v>75</v>
+        <v>39</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>76</v>
+        <v>40</v>
       </c>
       <c r="C1" s="8" t="s">
-        <v>77</v>
+        <v>41</v>
       </c>
       <c r="D1" s="8" t="s">
-        <v>78</v>
+        <v>42</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1479,13 +1181,13 @@
         <v>2090142</v>
       </c>
       <c r="B2" t="s">
-        <v>79</v>
+        <v>62</v>
       </c>
       <c r="C2" t="s">
-        <v>80</v>
+        <v>43</v>
       </c>
       <c r="D2" t="s">
-        <v>81</v>
+        <v>44</v>
       </c>
     </row>
     <row r="28" ht="14.4" x14ac:dyDescent="0.3"/>
@@ -1532,26 +1234,26 @@
     <row r="58" spans="2:11" ht="14.4" x14ac:dyDescent="0.3"/>
     <row r="59" spans="2:11" ht="14.4" x14ac:dyDescent="0.3"/>
     <row r="60" spans="2:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="G60" s="14"/>
-      <c r="H60" s="14"/>
-      <c r="I60" s="14"/>
-      <c r="J60" s="14"/>
+      <c r="G60" s="13"/>
+      <c r="H60" s="13"/>
+      <c r="I60" s="13"/>
+      <c r="J60" s="13"/>
     </row>
     <row r="61" spans="2:11" ht="14.4" x14ac:dyDescent="0.3">
       <c r="G61" s="1"/>
       <c r="I61" s="1"/>
     </row>
     <row r="62" spans="2:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="H62" s="14"/>
-      <c r="I62" s="14"/>
-      <c r="J62" s="14"/>
-      <c r="K62" s="14"/>
+      <c r="H62" s="13"/>
+      <c r="I62" s="13"/>
+      <c r="J62" s="13"/>
+      <c r="K62" s="13"/>
     </row>
     <row r="63" spans="2:11" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="H63" s="14"/>
-      <c r="I63" s="14"/>
-      <c r="J63" s="14"/>
-      <c r="K63" s="14"/>
+      <c r="H63" s="13"/>
+      <c r="I63" s="13"/>
+      <c r="J63" s="13"/>
+      <c r="K63" s="13"/>
     </row>
     <row r="64" spans="2:11" ht="14.4" x14ac:dyDescent="0.3"/>
     <row r="65" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
@@ -1617,7 +1319,7 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C5"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="22.77734375" customWidth="1"/>
@@ -1627,10 +1329,10 @@
   <sheetData>
     <row r="1" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
-        <v>82</v>
+        <v>45</v>
       </c>
       <c r="B1" s="8" t="s">
-        <v>76</v>
+        <v>40</v>
       </c>
       <c r="C1" s="8" t="s">
         <v>2</v>
@@ -1638,79 +1340,46 @@
     </row>
     <row r="2" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
-        <v>83</v>
+        <v>63</v>
       </c>
       <c r="B2" t="s">
-        <v>84</v>
+        <v>66</v>
       </c>
       <c r="C2" t="s">
-        <v>85</v>
+        <v>68</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>86</v>
+        <v>64</v>
       </c>
       <c r="B3" t="s">
-        <v>87</v>
+        <v>66</v>
       </c>
       <c r="C3" t="s">
-        <v>14</v>
+        <v>68</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>88</v>
+        <v>65</v>
       </c>
       <c r="B4" t="s">
-        <v>89</v>
+        <v>66</v>
       </c>
       <c r="C4" t="s">
-        <v>90</v>
+        <v>68</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>91</v>
+        <v>46</v>
       </c>
       <c r="B5" t="s">
-        <v>92</v>
+        <v>67</v>
       </c>
       <c r="C5" t="s">
-        <v>93</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" t="s">
-        <v>94</v>
-      </c>
-      <c r="B6" t="s">
-        <v>95</v>
-      </c>
-      <c r="C6" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" t="s">
-        <v>97</v>
-      </c>
-      <c r="B7" t="s">
-        <v>98</v>
-      </c>
-      <c r="C7" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" t="s">
-        <v>100</v>
-      </c>
-      <c r="B8" t="s">
-        <v>101</v>
-      </c>
-      <c r="C8" t="s">
-        <v>44</v>
+        <v>69</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sektionsnummer bei Gruppen korrigiert
</commit_message>
<xml_diff>
--- a/Keys.xlsx
+++ b/Keys.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Berenike\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ED840244-9C18-4BA5-A67C-1EB4612D048A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7305627-DED4-4B9E-9F1A-3B4638F877CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -232,12 +232,6 @@
     <t>Familienwanderung</t>
   </si>
   <si>
-    <t>/267 - Sektion Trier/Gruppen/Wandergruppe</t>
-  </si>
-  <si>
-    <t>/267 - Sektion Trier/Gruppen/Mountainbiken</t>
-  </si>
-  <si>
     <t>Sektionsabend</t>
   </si>
   <si>
@@ -247,25 +241,31 @@
     <t>Mountaindogs</t>
   </si>
   <si>
-    <t>/267 - Sektion Trier/Gruppen/Mountaindogs</t>
-  </si>
-  <si>
     <t>MTD</t>
   </si>
   <si>
     <t>Leistungskader</t>
   </si>
   <si>
-    <t>/267 - Sektion Trier/Gruppen/Klettern</t>
-  </si>
-  <si>
-    <t>/267 - Sektion Trier/Gruppen/Bergsteigen</t>
-  </si>
-  <si>
-    <t>/267 - Sektion Trier/Gruppen/Leistungskader</t>
-  </si>
-  <si>
     <t>WA</t>
+  </si>
+  <si>
+    <t>/264 - Sektion Trier/Gruppen/Wandergruppe</t>
+  </si>
+  <si>
+    <t>/264 - Sektion Trier/Gruppen/Mountainbiken</t>
+  </si>
+  <si>
+    <t>/264 - Sektion Trier/Gruppen/Mountaindogs</t>
+  </si>
+  <si>
+    <t>/264 - Sektion Trier/Gruppen/Klettern</t>
+  </si>
+  <si>
+    <t>/264 - Sektion Trier/Gruppen/Bergsteigen</t>
+  </si>
+  <si>
+    <t>/264 - Sektion Trier/Gruppen/Leistungskader</t>
   </si>
 </sst>
 </file>
@@ -1367,10 +1367,10 @@
         <v>63</v>
       </c>
       <c r="B2" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C2" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1378,10 +1378,10 @@
         <v>64</v>
       </c>
       <c r="B3" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C3" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1389,10 +1389,10 @@
         <v>65</v>
       </c>
       <c r="B4" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="C4" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1400,7 +1400,7 @@
         <v>46</v>
       </c>
       <c r="B5" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="C5" t="s">
         <v>7</v>
@@ -1408,23 +1408,23 @@
     </row>
     <row r="6" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B8" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="C8" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
@@ -1432,7 +1432,7 @@
         <v>50</v>
       </c>
       <c r="B9" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C9" t="s">
         <v>61</v>
@@ -1443,7 +1443,7 @@
         <v>47</v>
       </c>
       <c r="B10" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="C10" t="s">
         <v>59</v>
@@ -1451,10 +1451,10 @@
     </row>
     <row r="11" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="B11" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="C11" t="s">
         <v>58</v>

</xml_diff>

<commit_message>
Veranstaltungen zu Kategorie hinzugefügt
</commit_message>
<xml_diff>
--- a/Keys.xlsx
+++ b/Keys.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Berenike\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pl/git/github/PhilippLemke/DAV360_Transformator/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D7305627-DED4-4B9E-9F1A-3B4638F877CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F65B5270-5B2A-1445-B818-B4D6FEA3538B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="20180" windowHeight="12460" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Kategorie" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="102" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="80">
   <si>
     <t>ID</t>
   </si>
@@ -266,13 +266,19 @@
   </si>
   <si>
     <t>/264 - Sektion Trier/Gruppen/Leistungskader</t>
+  </si>
+  <si>
+    <t>Veranstaltung</t>
+  </si>
+  <si>
+    <t>VA</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -299,6 +305,12 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -320,7 +332,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -351,9 +363,10 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -613,15 +626,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C1048576"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.5" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.44140625" style="3"/>
-    <col min="2" max="2" width="36.109375" style="3" customWidth="1"/>
+    <col min="1" max="1" width="10.5" style="3"/>
+    <col min="2" max="2" width="36.1640625" style="3" customWidth="1"/>
     <col min="3" max="3" width="13" customWidth="1"/>
     <col min="4" max="4" width="16.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -632,7 +645,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>417</v>
       </c>
@@ -643,7 +656,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>418</v>
       </c>
@@ -654,7 +667,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>419</v>
       </c>
@@ -665,7 +678,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>420</v>
       </c>
@@ -676,7 +689,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>421</v>
       </c>
@@ -687,7 +700,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>422</v>
       </c>
@@ -698,7 +711,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>423</v>
       </c>
@@ -709,7 +722,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>35246</v>
       </c>
@@ -720,7 +733,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>424</v>
       </c>
@@ -731,7 +744,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>871</v>
       </c>
@@ -742,7 +755,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>22965</v>
       </c>
@@ -753,7 +766,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>425</v>
       </c>
@@ -764,7 +777,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="14" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>426</v>
       </c>
@@ -775,7 +788,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>2284</v>
       </c>
@@ -786,7 +799,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="16" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>39348</v>
       </c>
@@ -797,52 +810,59 @@
         <v>58</v>
       </c>
     </row>
-    <row r="17" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A17"/>
-      <c r="B17"/>
-    </row>
-    <row r="18" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A17">
+        <v>12345</v>
+      </c>
+      <c r="B17" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="C17" s="14" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A18"/>
       <c r="B18"/>
     </row>
-    <row r="19" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A19"/>
       <c r="B19"/>
     </row>
-    <row r="20" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A20"/>
       <c r="B20"/>
     </row>
-    <row r="21" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A21"/>
       <c r="B21"/>
     </row>
-    <row r="22" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A22"/>
       <c r="B22"/>
     </row>
-    <row r="23" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A23"/>
       <c r="B23"/>
     </row>
-    <row r="24" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A24"/>
       <c r="B24"/>
     </row>
-    <row r="25" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A25"/>
       <c r="B25"/>
     </row>
-    <row r="26" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A26"/>
       <c r="B26"/>
     </row>
-    <row r="27" spans="1:2" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
       <c r="B27"/>
     </row>
-    <row r="1048574" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="1048575" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="1048576" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="1048574" x14ac:dyDescent="0.2"/>
+    <row r="1048575" x14ac:dyDescent="0.2"/>
+    <row r="1048576" x14ac:dyDescent="0.2"/>
   </sheetData>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -856,13 +876,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.5" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.44140625" style="3"/>
-    <col min="2" max="2" width="13.77734375" style="3" customWidth="1"/>
+    <col min="1" max="1" width="10.5" style="3"/>
+    <col min="2" max="2" width="13.83203125" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -870,7 +890,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="3">
         <v>413</v>
       </c>
@@ -878,7 +898,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="3">
         <v>414</v>
       </c>
@@ -886,7 +906,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
         <v>415</v>
       </c>
@@ -894,7 +914,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="3">
         <v>416</v>
       </c>
@@ -915,13 +935,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.5" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.44140625" style="3"/>
+    <col min="1" max="1" width="10.5" style="3"/>
     <col min="2" max="2" width="12.6640625" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -929,7 +949,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="3">
         <v>409</v>
       </c>
@@ -937,7 +957,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="3">
         <v>410</v>
       </c>
@@ -945,7 +965,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
         <v>411</v>
       </c>
@@ -953,7 +973,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="3">
         <v>412</v>
       </c>
@@ -974,13 +994,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.5" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="10.44140625" style="3"/>
+    <col min="1" max="1" width="10.5" style="3"/>
     <col min="2" max="2" width="13.33203125" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -988,7 +1008,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="3">
         <v>405</v>
       </c>
@@ -996,7 +1016,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="3">
         <v>406</v>
       </c>
@@ -1004,7 +1024,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
         <v>407</v>
       </c>
@@ -1012,7 +1032,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="3">
         <v>408</v>
       </c>
@@ -1033,13 +1053,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.5" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="17" style="3" customWidth="1"/>
-    <col min="2" max="2" width="55.109375" customWidth="1"/>
+    <col min="2" max="2" width="55.1640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -1047,7 +1067,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="3">
         <v>392</v>
       </c>
@@ -1056,7 +1076,7 @@
       </c>
       <c r="C2" s="12"/>
     </row>
-    <row r="3" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A3" s="3">
         <v>393</v>
       </c>
@@ -1064,7 +1084,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A4" s="3">
         <v>394</v>
       </c>
@@ -1072,7 +1092,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A5" s="3">
         <v>395</v>
       </c>
@@ -1080,7 +1100,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A6" s="3">
         <v>396</v>
       </c>
@@ -1088,7 +1108,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" ht="16" x14ac:dyDescent="0.2">
       <c r="A7" s="3">
         <v>48744</v>
       </c>
@@ -1096,7 +1116,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A8" s="3">
         <v>48745</v>
       </c>
@@ -1104,7 +1124,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A9" s="3">
         <v>48746</v>
       </c>
@@ -1128,13 +1148,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.5" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="14.109375" customWidth="1"/>
-    <col min="2" max="2" width="20.44140625" customWidth="1"/>
+    <col min="1" max="1" width="14.1640625" customWidth="1"/>
+    <col min="2" max="2" width="20.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -1142,7 +1162,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>397</v>
       </c>
@@ -1150,7 +1170,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>398</v>
       </c>
@@ -1158,7 +1178,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>39481</v>
       </c>
@@ -1179,14 +1199,14 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:K1048576"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.5" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="12" style="3" customWidth="1"/>
-    <col min="2" max="2" width="74.109375" customWidth="1"/>
+    <col min="2" max="2" width="74.1640625" customWidth="1"/>
     <col min="3" max="3" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" s="7" t="s">
         <v>39</v>
       </c>
@@ -1200,7 +1220,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="3">
         <v>2090142</v>
       </c>
@@ -1214,94 +1234,94 @@
         <v>44</v>
       </c>
     </row>
-    <row r="28" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="29" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="30" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="31" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="32" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="33" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="34" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="35" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="36" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="37" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="38" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="39" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="40" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="41" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="42" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="43" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="44" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="45" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="46" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="47" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="48" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="49" spans="2:11" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="50" spans="2:11" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="28" x14ac:dyDescent="0.2"/>
+    <row r="29" x14ac:dyDescent="0.2"/>
+    <row r="30" x14ac:dyDescent="0.2"/>
+    <row r="31" x14ac:dyDescent="0.2"/>
+    <row r="32" x14ac:dyDescent="0.2"/>
+    <row r="33" x14ac:dyDescent="0.2"/>
+    <row r="34" x14ac:dyDescent="0.2"/>
+    <row r="35" x14ac:dyDescent="0.2"/>
+    <row r="36" x14ac:dyDescent="0.2"/>
+    <row r="37" x14ac:dyDescent="0.2"/>
+    <row r="38" x14ac:dyDescent="0.2"/>
+    <row r="39" x14ac:dyDescent="0.2"/>
+    <row r="40" x14ac:dyDescent="0.2"/>
+    <row r="41" x14ac:dyDescent="0.2"/>
+    <row r="42" x14ac:dyDescent="0.2"/>
+    <row r="43" x14ac:dyDescent="0.2"/>
+    <row r="44" x14ac:dyDescent="0.2"/>
+    <row r="45" x14ac:dyDescent="0.2"/>
+    <row r="46" x14ac:dyDescent="0.2"/>
+    <row r="47" x14ac:dyDescent="0.2"/>
+    <row r="48" x14ac:dyDescent="0.2"/>
+    <row r="49" spans="2:11" x14ac:dyDescent="0.2"/>
+    <row r="50" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B50" s="2"/>
     </row>
-    <row r="51" spans="2:11" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="52" spans="2:11" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="53" spans="2:11" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="54" spans="2:11" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="55" spans="2:11" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="51" spans="2:11" x14ac:dyDescent="0.2"/>
+    <row r="52" spans="2:11" x14ac:dyDescent="0.2"/>
+    <row r="53" spans="2:11" x14ac:dyDescent="0.2"/>
+    <row r="54" spans="2:11" x14ac:dyDescent="0.2"/>
+    <row r="55" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B55" s="9"/>
       <c r="C55" s="9"/>
       <c r="D55" s="9"/>
     </row>
-    <row r="56" spans="2:11" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="57" spans="2:11" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="56" spans="2:11" x14ac:dyDescent="0.2"/>
+    <row r="57" spans="2:11" x14ac:dyDescent="0.2">
       <c r="B57" s="2"/>
       <c r="E57" s="1"/>
       <c r="F57" s="2"/>
       <c r="G57" s="2"/>
     </row>
-    <row r="58" spans="2:11" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="59" spans="2:11" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="60" spans="2:11" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="58" spans="2:11" x14ac:dyDescent="0.2"/>
+    <row r="59" spans="2:11" x14ac:dyDescent="0.2"/>
+    <row r="60" spans="2:11" x14ac:dyDescent="0.2">
       <c r="G60" s="13"/>
       <c r="H60" s="13"/>
       <c r="I60" s="13"/>
       <c r="J60" s="13"/>
     </row>
-    <row r="61" spans="2:11" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="61" spans="2:11" x14ac:dyDescent="0.2">
       <c r="G61" s="1"/>
       <c r="I61" s="1"/>
     </row>
-    <row r="62" spans="2:11" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="62" spans="2:11" x14ac:dyDescent="0.2">
       <c r="H62" s="13"/>
       <c r="I62" s="13"/>
       <c r="J62" s="13"/>
       <c r="K62" s="13"/>
     </row>
-    <row r="63" spans="2:11" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="63" spans="2:11" x14ac:dyDescent="0.2">
       <c r="H63" s="13"/>
       <c r="I63" s="13"/>
       <c r="J63" s="13"/>
       <c r="K63" s="13"/>
     </row>
-    <row r="64" spans="2:11" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="65" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="64" spans="2:11" x14ac:dyDescent="0.2"/>
+    <row r="65" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B65" s="9"/>
     </row>
-    <row r="66" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.2">
       <c r="B66" s="10"/>
     </row>
-    <row r="67" spans="1:7" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="68" spans="1:7" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="69" spans="1:7" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="70" spans="1:7" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="71" spans="1:7" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="72" spans="1:7" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="73" spans="1:7" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="74" spans="1:7" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="75" spans="1:7" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="76" spans="1:7" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="77" spans="1:7" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="78" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.2"/>
+    <row r="68" spans="1:7" x14ac:dyDescent="0.2"/>
+    <row r="69" spans="1:7" x14ac:dyDescent="0.2"/>
+    <row r="70" spans="1:7" x14ac:dyDescent="0.2"/>
+    <row r="71" spans="1:7" x14ac:dyDescent="0.2"/>
+    <row r="72" spans="1:7" x14ac:dyDescent="0.2"/>
+    <row r="73" spans="1:7" x14ac:dyDescent="0.2"/>
+    <row r="74" spans="1:7" x14ac:dyDescent="0.2"/>
+    <row r="75" spans="1:7" x14ac:dyDescent="0.2"/>
+    <row r="76" spans="1:7" x14ac:dyDescent="0.2"/>
+    <row r="77" spans="1:7" x14ac:dyDescent="0.2"/>
+    <row r="78" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A78" s="6"/>
       <c r="B78" s="2"/>
     </row>
-    <row r="79" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A79" s="6"/>
       <c r="B79" s="2"/>
       <c r="C79" s="2"/>
@@ -1310,19 +1330,19 @@
       <c r="F79" s="2"/>
       <c r="G79" s="2"/>
     </row>
-    <row r="80" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A80" s="6"/>
       <c r="B80" s="2"/>
       <c r="C80" s="2"/>
       <c r="D80" s="2"/>
       <c r="E80" s="11"/>
     </row>
-    <row r="1048571" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="1048572" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="1048573" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="1048574" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="1048575" ht="14.4" x14ac:dyDescent="0.3"/>
-    <row r="1048576" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="1048571" x14ac:dyDescent="0.2"/>
+    <row r="1048572" x14ac:dyDescent="0.2"/>
+    <row r="1048573" x14ac:dyDescent="0.2"/>
+    <row r="1048574" x14ac:dyDescent="0.2"/>
+    <row r="1048575" x14ac:dyDescent="0.2"/>
+    <row r="1048576" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="G60:H60"/>
@@ -1344,14 +1364,14 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:C11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="22.77734375" customWidth="1"/>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="107.33203125" customWidth="1"/>
-    <col min="3" max="3" width="26.44140625" customWidth="1"/>
+    <col min="3" max="3" width="26.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>45</v>
       </c>
@@ -1362,7 +1382,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>63</v>
       </c>
@@ -1373,7 +1393,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>64</v>
       </c>
@@ -1384,7 +1404,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>65</v>
       </c>
@@ -1395,7 +1415,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>46</v>
       </c>
@@ -1406,17 +1426,17 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>67</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>68</v>
       </c>
@@ -1427,7 +1447,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>50</v>
       </c>
@@ -1438,7 +1458,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>47</v>
       </c>
@@ -1449,7 +1469,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="11" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>70</v>
       </c>

</xml_diff>

<commit_message>
TeaserImage Pfad bei Gruppen ergaenzt
</commit_message>
<xml_diff>
--- a/Keys.xlsx
+++ b/Keys.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10419"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pl/git/github/PhilippLemke/DAV360_Transformator/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Berenike\DAV360_Transformator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F65B5270-5B2A-1445-B818-B4D6FEA3538B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E88B1EE-F2FD-4A3F-A925-1AE841F09DEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="20180" windowHeight="12460" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Kategorie" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="91">
   <si>
     <t>ID</t>
   </si>
@@ -272,13 +272,46 @@
   </si>
   <si>
     <t>VA</t>
+  </si>
+  <si>
+    <t>/264 - Sektion Trier/Events/Pausenplatz.jpg</t>
+  </si>
+  <si>
+    <t>/264 - Sektion Trier/Events/Sonntagswanderung.jpg</t>
+  </si>
+  <si>
+    <t>/264 - Sektion Trier/Events/Familienwanderung.jpg</t>
+  </si>
+  <si>
+    <t>/264 - Sektion Trier/Events/Mountainbike.jpg</t>
+  </si>
+  <si>
+    <t>/264 - Sektion Trier/Events/Kaminfeuer.jpg</t>
+  </si>
+  <si>
+    <t>/264 - Sektion Trier/Events/Arbeitstag.jpg</t>
+  </si>
+  <si>
+    <t>/264 - Sektion Trier/Gruppen/Mountaindogs1.jpg</t>
+  </si>
+  <si>
+    <t>/264 - Sektion Trier/Gruppen/Klettern.jpg</t>
+  </si>
+  <si>
+    <t>/264 - Sektion Trier/Gruppen/Bergsteigen.jpg</t>
+  </si>
+  <si>
+    <t>/264 - Sektion Trier/Gruppen/Leistungskader.jpg</t>
+  </si>
+  <si>
+    <t>Image_path</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -311,6 +344,12 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -332,7 +371,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -359,14 +398,15 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -626,15 +666,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:C1048576"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.5" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.5" style="3"/>
-    <col min="2" max="2" width="36.1640625" style="3" customWidth="1"/>
+    <col min="1" max="1" width="10.44140625" style="3"/>
+    <col min="2" max="2" width="36.109375" style="3" customWidth="1"/>
     <col min="3" max="3" width="13" customWidth="1"/>
     <col min="4" max="4" width="16.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -645,7 +685,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>417</v>
       </c>
@@ -656,7 +696,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>418</v>
       </c>
@@ -667,7 +707,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>419</v>
       </c>
@@ -678,7 +718,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A5">
         <v>420</v>
       </c>
@@ -689,7 +729,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A6">
         <v>421</v>
       </c>
@@ -700,7 +740,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A7">
         <v>422</v>
       </c>
@@ -711,7 +751,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A8">
         <v>423</v>
       </c>
@@ -722,7 +762,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A9">
         <v>35246</v>
       </c>
@@ -733,7 +773,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A10">
         <v>424</v>
       </c>
@@ -744,7 +784,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A11">
         <v>871</v>
       </c>
@@ -755,7 +795,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A12">
         <v>22965</v>
       </c>
@@ -766,7 +806,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A13">
         <v>425</v>
       </c>
@@ -777,7 +817,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A14">
         <v>426</v>
       </c>
@@ -788,7 +828,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A15">
         <v>2284</v>
       </c>
@@ -799,7 +839,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A16">
         <v>39348</v>
       </c>
@@ -810,59 +850,57 @@
         <v>58</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A17">
-        <v>12345</v>
-      </c>
-      <c r="B17" s="14" t="s">
+    <row r="17" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A17"/>
+      <c r="B17" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="C17" s="14" t="s">
+      <c r="C17" s="12" t="s">
         <v>79</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A18"/>
       <c r="B18"/>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A19"/>
       <c r="B19"/>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A20"/>
       <c r="B20"/>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A21"/>
       <c r="B21"/>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A22"/>
       <c r="B22"/>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A23"/>
       <c r="B23"/>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A24"/>
       <c r="B24"/>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A25"/>
       <c r="B25"/>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A26"/>
       <c r="B26"/>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B27"/>
     </row>
-    <row r="1048574" x14ac:dyDescent="0.2"/>
-    <row r="1048575" x14ac:dyDescent="0.2"/>
-    <row r="1048576" x14ac:dyDescent="0.2"/>
+    <row r="1048574" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="1048575" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="1048576" ht="14.4" x14ac:dyDescent="0.3"/>
   </sheetData>
   <pageMargins left="0.78749999999999998" right="0.78749999999999998" top="1.05277777777778" bottom="1.05277777777778" header="0.78749999999999998" footer="0.78749999999999998"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -876,13 +914,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.5" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.5" style="3"/>
-    <col min="2" max="2" width="13.83203125" style="3" customWidth="1"/>
+    <col min="1" max="1" width="10.44140625" style="3"/>
+    <col min="2" max="2" width="13.77734375" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -890,7 +928,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3">
         <v>413</v>
       </c>
@@ -898,7 +936,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3">
         <v>414</v>
       </c>
@@ -906,7 +944,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3">
         <v>415</v>
       </c>
@@ -914,7 +952,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3">
         <v>416</v>
       </c>
@@ -935,13 +973,13 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.5" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.5" style="3"/>
+    <col min="1" max="1" width="10.44140625" style="3"/>
     <col min="2" max="2" width="12.6640625" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -949,7 +987,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3">
         <v>409</v>
       </c>
@@ -957,7 +995,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3">
         <v>410</v>
       </c>
@@ -965,7 +1003,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3">
         <v>411</v>
       </c>
@@ -973,7 +1011,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3">
         <v>412</v>
       </c>
@@ -994,13 +1032,13 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:B5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.5" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="10.5" style="3"/>
+    <col min="1" max="1" width="10.44140625" style="3"/>
     <col min="2" max="2" width="13.33203125" style="3" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -1008,7 +1046,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3">
         <v>405</v>
       </c>
@@ -1016,7 +1054,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="3">
         <v>406</v>
       </c>
@@ -1024,7 +1062,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" s="3">
         <v>407</v>
       </c>
@@ -1032,7 +1070,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3">
         <v>408</v>
       </c>
@@ -1053,13 +1091,13 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:C9"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.5" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="17" style="3" customWidth="1"/>
-    <col min="2" max="2" width="55.1640625" customWidth="1"/>
+    <col min="2" max="2" width="55.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -1067,16 +1105,16 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:3" ht="13.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3">
         <v>392</v>
       </c>
-      <c r="B2" s="12" t="s">
+      <c r="B2" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="C2" s="12"/>
-    </row>
-    <row r="3" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+      <c r="C2" s="14"/>
+    </row>
+    <row r="3" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A3" s="3">
         <v>393</v>
       </c>
@@ -1084,7 +1122,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A4" s="3">
         <v>394</v>
       </c>
@@ -1092,7 +1130,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A5" s="3">
         <v>395</v>
       </c>
@@ -1100,7 +1138,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A6" s="3">
         <v>396</v>
       </c>
@@ -1108,7 +1146,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="16" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A7" s="3">
         <v>48744</v>
       </c>
@@ -1116,7 +1154,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A8" s="3">
         <v>48745</v>
       </c>
@@ -1124,7 +1162,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A9" s="3">
         <v>48746</v>
       </c>
@@ -1148,13 +1186,13 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.5" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="14.1640625" customWidth="1"/>
-    <col min="2" max="2" width="20.5" customWidth="1"/>
+    <col min="1" max="1" width="14.109375" customWidth="1"/>
+    <col min="2" max="2" width="20.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -1162,7 +1200,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>397</v>
       </c>
@@ -1170,7 +1208,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="3" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3">
         <v>398</v>
       </c>
@@ -1178,7 +1216,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:2" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4">
         <v>39481</v>
       </c>
@@ -1199,14 +1237,14 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:K1048576"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.5" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.44140625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12" style="3" customWidth="1"/>
-    <col min="2" max="2" width="74.1640625" customWidth="1"/>
+    <col min="2" max="2" width="74.109375" customWidth="1"/>
     <col min="3" max="3" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
         <v>39</v>
       </c>
@@ -1220,7 +1258,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="3">
         <v>2090142</v>
       </c>
@@ -1234,94 +1272,94 @@
         <v>44</v>
       </c>
     </row>
-    <row r="28" x14ac:dyDescent="0.2"/>
-    <row r="29" x14ac:dyDescent="0.2"/>
-    <row r="30" x14ac:dyDescent="0.2"/>
-    <row r="31" x14ac:dyDescent="0.2"/>
-    <row r="32" x14ac:dyDescent="0.2"/>
-    <row r="33" x14ac:dyDescent="0.2"/>
-    <row r="34" x14ac:dyDescent="0.2"/>
-    <row r="35" x14ac:dyDescent="0.2"/>
-    <row r="36" x14ac:dyDescent="0.2"/>
-    <row r="37" x14ac:dyDescent="0.2"/>
-    <row r="38" x14ac:dyDescent="0.2"/>
-    <row r="39" x14ac:dyDescent="0.2"/>
-    <row r="40" x14ac:dyDescent="0.2"/>
-    <row r="41" x14ac:dyDescent="0.2"/>
-    <row r="42" x14ac:dyDescent="0.2"/>
-    <row r="43" x14ac:dyDescent="0.2"/>
-    <row r="44" x14ac:dyDescent="0.2"/>
-    <row r="45" x14ac:dyDescent="0.2"/>
-    <row r="46" x14ac:dyDescent="0.2"/>
-    <row r="47" x14ac:dyDescent="0.2"/>
-    <row r="48" x14ac:dyDescent="0.2"/>
-    <row r="49" spans="2:11" x14ac:dyDescent="0.2"/>
-    <row r="50" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="28" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="29" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="30" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="31" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="32" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="33" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="34" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="35" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="36" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="37" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="38" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="39" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="40" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="41" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="42" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="43" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="44" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="45" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="46" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="47" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="48" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="49" spans="2:11" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="50" spans="2:11" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B50" s="2"/>
     </row>
-    <row r="51" spans="2:11" x14ac:dyDescent="0.2"/>
-    <row r="52" spans="2:11" x14ac:dyDescent="0.2"/>
-    <row r="53" spans="2:11" x14ac:dyDescent="0.2"/>
-    <row r="54" spans="2:11" x14ac:dyDescent="0.2"/>
-    <row r="55" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="51" spans="2:11" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="52" spans="2:11" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="53" spans="2:11" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="54" spans="2:11" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="55" spans="2:11" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B55" s="9"/>
       <c r="C55" s="9"/>
       <c r="D55" s="9"/>
     </row>
-    <row r="56" spans="2:11" x14ac:dyDescent="0.2"/>
-    <row r="57" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="56" spans="2:11" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="57" spans="2:11" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B57" s="2"/>
       <c r="E57" s="1"/>
       <c r="F57" s="2"/>
       <c r="G57" s="2"/>
     </row>
-    <row r="58" spans="2:11" x14ac:dyDescent="0.2"/>
-    <row r="59" spans="2:11" x14ac:dyDescent="0.2"/>
-    <row r="60" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="G60" s="13"/>
-      <c r="H60" s="13"/>
-      <c r="I60" s="13"/>
-      <c r="J60" s="13"/>
-    </row>
-    <row r="61" spans="2:11" x14ac:dyDescent="0.2">
+    <row r="58" spans="2:11" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="59" spans="2:11" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="60" spans="2:11" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="G60" s="15"/>
+      <c r="H60" s="15"/>
+      <c r="I60" s="15"/>
+      <c r="J60" s="15"/>
+    </row>
+    <row r="61" spans="2:11" ht="14.4" x14ac:dyDescent="0.3">
       <c r="G61" s="1"/>
       <c r="I61" s="1"/>
     </row>
-    <row r="62" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="H62" s="13"/>
-      <c r="I62" s="13"/>
-      <c r="J62" s="13"/>
-      <c r="K62" s="13"/>
-    </row>
-    <row r="63" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="H63" s="13"/>
-      <c r="I63" s="13"/>
-      <c r="J63" s="13"/>
-      <c r="K63" s="13"/>
-    </row>
-    <row r="64" spans="2:11" x14ac:dyDescent="0.2"/>
-    <row r="65" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="62" spans="2:11" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="H62" s="15"/>
+      <c r="I62" s="15"/>
+      <c r="J62" s="15"/>
+      <c r="K62" s="15"/>
+    </row>
+    <row r="63" spans="2:11" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="H63" s="15"/>
+      <c r="I63" s="15"/>
+      <c r="J63" s="15"/>
+      <c r="K63" s="15"/>
+    </row>
+    <row r="64" spans="2:11" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="65" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B65" s="9"/>
     </row>
-    <row r="66" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
       <c r="B66" s="10"/>
     </row>
-    <row r="67" spans="1:7" x14ac:dyDescent="0.2"/>
-    <row r="68" spans="1:7" x14ac:dyDescent="0.2"/>
-    <row r="69" spans="1:7" x14ac:dyDescent="0.2"/>
-    <row r="70" spans="1:7" x14ac:dyDescent="0.2"/>
-    <row r="71" spans="1:7" x14ac:dyDescent="0.2"/>
-    <row r="72" spans="1:7" x14ac:dyDescent="0.2"/>
-    <row r="73" spans="1:7" x14ac:dyDescent="0.2"/>
-    <row r="74" spans="1:7" x14ac:dyDescent="0.2"/>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.2"/>
-    <row r="76" spans="1:7" x14ac:dyDescent="0.2"/>
-    <row r="77" spans="1:7" x14ac:dyDescent="0.2"/>
-    <row r="78" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:7" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="68" spans="1:7" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="69" spans="1:7" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="70" spans="1:7" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="71" spans="1:7" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="72" spans="1:7" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="73" spans="1:7" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="74" spans="1:7" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="75" spans="1:7" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="76" spans="1:7" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="77" spans="1:7" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="78" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A78" s="6"/>
       <c r="B78" s="2"/>
     </row>
-    <row r="79" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A79" s="6"/>
       <c r="B79" s="2"/>
       <c r="C79" s="2"/>
@@ -1330,19 +1368,19 @@
       <c r="F79" s="2"/>
       <c r="G79" s="2"/>
     </row>
-    <row r="80" spans="1:7" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:7" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A80" s="6"/>
       <c r="B80" s="2"/>
       <c r="C80" s="2"/>
       <c r="D80" s="2"/>
       <c r="E80" s="11"/>
     </row>
-    <row r="1048571" x14ac:dyDescent="0.2"/>
-    <row r="1048572" x14ac:dyDescent="0.2"/>
-    <row r="1048573" x14ac:dyDescent="0.2"/>
-    <row r="1048574" x14ac:dyDescent="0.2"/>
-    <row r="1048575" x14ac:dyDescent="0.2"/>
-    <row r="1048576" x14ac:dyDescent="0.2"/>
+    <row r="1048571" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="1048572" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="1048573" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="1048574" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="1048575" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="1048576" ht="14.4" x14ac:dyDescent="0.3"/>
   </sheetData>
   <mergeCells count="6">
     <mergeCell ref="G60:H60"/>
@@ -1363,15 +1401,15 @@
 
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
-  <dimension ref="A1:C11"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:D11"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="1" max="1" width="22.77734375" customWidth="1"/>
     <col min="2" max="2" width="107.33203125" customWidth="1"/>
-    <col min="3" max="3" width="26.5" customWidth="1"/>
+    <col min="3" max="3" width="26.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>45</v>
       </c>
@@ -1381,8 +1419,11 @@
       <c r="C1" s="8" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="2" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D1" s="13" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>63</v>
       </c>
@@ -1392,8 +1433,11 @@
       <c r="C2" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="3" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D2" s="12" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>64</v>
       </c>
@@ -1403,8 +1447,11 @@
       <c r="C3" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="4" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D3" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>65</v>
       </c>
@@ -1414,8 +1461,11 @@
       <c r="C4" t="s">
         <v>71</v>
       </c>
-    </row>
-    <row r="5" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D4" s="12" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>46</v>
       </c>
@@ -1425,18 +1475,27 @@
       <c r="C5" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="6" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D5" s="12" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="7" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D6" s="12" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>67</v>
       </c>
-    </row>
-    <row r="8" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D7" s="12" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>68</v>
       </c>
@@ -1446,8 +1505,11 @@
       <c r="C8" t="s">
         <v>69</v>
       </c>
-    </row>
-    <row r="9" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D8" s="12" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>50</v>
       </c>
@@ -1457,8 +1519,11 @@
       <c r="C9" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="10" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D9" s="12" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>47</v>
       </c>
@@ -1468,8 +1533,11 @@
       <c r="C10" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="11" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D10" s="12" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>70</v>
       </c>
@@ -1479,9 +1547,12 @@
       <c r="C11" t="s">
         <v>58</v>
       </c>
+      <c r="D11" s="12" t="s">
+        <v>89</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Kategorie (Houchtour) Hochtouren ergänzt
</commit_message>
<xml_diff>
--- a/Keys.xlsx
+++ b/Keys.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Berenike\DAV360_Transformator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1E88B1EE-F2FD-4A3F-A925-1AE841F09DEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1316BFFD-3153-4202-8F5A-7E6FC79A2B15}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" firstSheet="2" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Kategorie" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="117" uniqueCount="92">
   <si>
     <t>ID</t>
   </si>
@@ -305,6 +305,9 @@
   </si>
   <si>
     <t>Image_path</t>
+  </si>
+  <si>
+    <t>Hochtour</t>
   </si>
 </sst>
 </file>
@@ -851,17 +854,24 @@
       </c>
     </row>
     <row r="17" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
-      <c r="A17"/>
-      <c r="B17" s="12" t="s">
-        <v>78</v>
-      </c>
-      <c r="C17" s="12" t="s">
-        <v>79</v>
+      <c r="A17">
+        <v>420</v>
+      </c>
+      <c r="B17" t="s">
+        <v>91</v>
+      </c>
+      <c r="C17" t="s">
+        <v>4</v>
       </c>
     </row>
     <row r="18" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A18"/>
-      <c r="B18"/>
+      <c r="B18" s="12" t="s">
+        <v>78</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="19" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
       <c r="A19"/>
@@ -896,9 +906,12 @@
       <c r="B26"/>
     </row>
     <row r="27" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="A27"/>
       <c r="B27"/>
     </row>
-    <row r="1048574" ht="14.4" x14ac:dyDescent="0.3"/>
+    <row r="28" spans="1:3" ht="14.4" x14ac:dyDescent="0.3">
+      <c r="B28"/>
+    </row>
     <row r="1048575" ht="14.4" x14ac:dyDescent="0.3"/>
     <row r="1048576" ht="14.4" x14ac:dyDescent="0.3"/>
   </sheetData>

</xml_diff>